<commit_message>
Require JSON re-scan and Excel verify before a complete file.
Sunday --fill-missing now fails on empty stats instead of mailing a sheet with blank fouls/corners/cards.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/predykcje_2026.xlsx
+++ b/predykcje_2026.xlsx
@@ -900,6 +900,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>13</v>
+      </c>
+      <c r="H5" t="n">
+        <v>17</v>
+      </c>
+      <c r="I5" t="n">
+        <v>30</v>
+      </c>
+      <c r="J5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>6</v>
+      </c>
+      <c r="R5" t="n">
+        <v>21</v>
+      </c>
+      <c r="S5" t="n">
+        <v>8</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -932,6 +977,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H6" t="n">
+        <v>11</v>
+      </c>
+      <c r="I6" t="n">
+        <v>29</v>
+      </c>
+      <c r="J6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" t="n">
+        <v>22</v>
+      </c>
+      <c r="S6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1426,6 +1516,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G13" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" t="n">
+        <v>9</v>
+      </c>
+      <c r="I13" t="n">
+        <v>16</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>10</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4</v>
+      </c>
+      <c r="P13" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>7</v>
+      </c>
+      <c r="R13" t="n">
+        <v>13</v>
+      </c>
+      <c r="S13" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" t="n">
+        <v>2</v>
+      </c>
+      <c r="U13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1535,6 +1670,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="n">
+        <v>11</v>
+      </c>
+      <c r="I15" t="n">
+        <v>21</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" t="n">
+        <v>15</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" t="n">
+        <v>5</v>
+      </c>
+      <c r="P15" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>18</v>
+      </c>
+      <c r="R15" t="n">
+        <v>32</v>
+      </c>
+      <c r="S15" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" t="n">
+        <v>5</v>
+      </c>
+      <c r="U15" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1798,6 +1978,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G19" t="n">
+        <v>13</v>
+      </c>
+      <c r="H19" t="n">
+        <v>16</v>
+      </c>
+      <c r="I19" t="n">
+        <v>29</v>
+      </c>
+      <c r="J19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>6</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>6</v>
+      </c>
+      <c r="P19" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>11</v>
+      </c>
+      <c r="R19" t="n">
+        <v>26</v>
+      </c>
+      <c r="S19" t="n">
+        <v>3</v>
+      </c>
+      <c r="T19" t="n">
+        <v>4</v>
+      </c>
+      <c r="U19" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1830,6 +2055,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" t="n">
+        <v>22</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>10</v>
+      </c>
+      <c r="L20" t="n">
+        <v>12</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" t="n">
+        <v>4</v>
+      </c>
+      <c r="P20" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>18</v>
+      </c>
+      <c r="R20" t="n">
+        <v>28</v>
+      </c>
+      <c r="S20" t="n">
+        <v>4</v>
+      </c>
+      <c r="T20" t="n">
+        <v>3</v>
+      </c>
+      <c r="U20" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1862,6 +2132,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G21" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" t="n">
+        <v>12</v>
+      </c>
+      <c r="I21" t="n">
+        <v>24</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K21" t="n">
+        <v>6</v>
+      </c>
+      <c r="L21" t="n">
+        <v>10</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" t="n">
+        <v>4</v>
+      </c>
+      <c r="O21" t="n">
+        <v>5</v>
+      </c>
+      <c r="P21" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>17</v>
+      </c>
+      <c r="R21" t="n">
+        <v>32</v>
+      </c>
+      <c r="S21" t="n">
+        <v>4</v>
+      </c>
+      <c r="T21" t="n">
+        <v>9</v>
+      </c>
+      <c r="U21" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1894,6 +2209,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G22" t="n">
+        <v>16</v>
+      </c>
+      <c r="H22" t="n">
+        <v>11</v>
+      </c>
+      <c r="I22" t="n">
+        <v>27</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5</v>
+      </c>
+      <c r="M22" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>5</v>
+      </c>
+      <c r="P22" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>7</v>
+      </c>
+      <c r="R22" t="n">
+        <v>16</v>
+      </c>
+      <c r="S22" t="n">
+        <v>5</v>
+      </c>
+      <c r="T22" t="n">
+        <v>3</v>
+      </c>
+      <c r="U22" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1926,6 +2286,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H23" t="n">
+        <v>12</v>
+      </c>
+      <c r="I23" t="n">
+        <v>22</v>
+      </c>
+      <c r="J23" t="n">
+        <v>10</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="n">
+        <v>11</v>
+      </c>
+      <c r="M23" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P23" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>4</v>
+      </c>
+      <c r="R23" t="n">
+        <v>34</v>
+      </c>
+      <c r="S23" t="n">
+        <v>13</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1958,6 +2363,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G24" t="n">
+        <v>9</v>
+      </c>
+      <c r="H24" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" t="n">
+        <v>17</v>
+      </c>
+      <c r="J24" t="n">
+        <v>10</v>
+      </c>
+      <c r="K24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L24" t="n">
+        <v>15</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>21</v>
+      </c>
+      <c r="R24" t="n">
+        <v>45</v>
+      </c>
+      <c r="S24" t="n">
+        <v>6</v>
+      </c>
+      <c r="T24" t="n">
+        <v>8</v>
+      </c>
+      <c r="U24" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2298,6 +2748,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G29" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" t="n">
+        <v>9</v>
+      </c>
+      <c r="I29" t="n">
+        <v>15</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" t="n">
+        <v>14</v>
+      </c>
+      <c r="L29" t="n">
+        <v>16</v>
+      </c>
+      <c r="M29" t="n">
+        <v>2</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>2</v>
+      </c>
+      <c r="P29" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>14</v>
+      </c>
+      <c r="R29" t="n">
+        <v>24</v>
+      </c>
+      <c r="S29" t="n">
+        <v>6</v>
+      </c>
+      <c r="T29" t="n">
+        <v>4</v>
+      </c>
+      <c r="U29" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2561,6 +3056,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G33" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" t="n">
+        <v>9</v>
+      </c>
+      <c r="J33" t="n">
+        <v>8</v>
+      </c>
+      <c r="K33" t="n">
+        <v>7</v>
+      </c>
+      <c r="L33" t="n">
+        <v>15</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O33" t="n">
+        <v>3</v>
+      </c>
+      <c r="P33" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>6</v>
+      </c>
+      <c r="R33" t="n">
+        <v>19</v>
+      </c>
+      <c r="S33" t="n">
+        <v>4</v>
+      </c>
+      <c r="T33" t="n">
+        <v>4</v>
+      </c>
+      <c r="U33" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2593,6 +3133,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G34" t="n">
+        <v>11</v>
+      </c>
+      <c r="H34" t="n">
+        <v>10</v>
+      </c>
+      <c r="I34" t="n">
+        <v>21</v>
+      </c>
+      <c r="J34" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" t="n">
+        <v>9</v>
+      </c>
+      <c r="L34" t="n">
+        <v>13</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>24</v>
+      </c>
+      <c r="R34" t="n">
+        <v>28</v>
+      </c>
+      <c r="S34" t="n">
+        <v>2</v>
+      </c>
+      <c r="T34" t="n">
+        <v>11</v>
+      </c>
+      <c r="U34" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2625,6 +3210,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G35" t="n">
+        <v>12</v>
+      </c>
+      <c r="H35" t="n">
+        <v>20</v>
+      </c>
+      <c r="I35" t="n">
+        <v>32</v>
+      </c>
+      <c r="J35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3</v>
+      </c>
+      <c r="L35" t="n">
+        <v>11</v>
+      </c>
+      <c r="M35" t="n">
+        <v>2</v>
+      </c>
+      <c r="N35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O35" t="n">
+        <v>5</v>
+      </c>
+      <c r="P35" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>5</v>
+      </c>
+      <c r="R35" t="n">
+        <v>19</v>
+      </c>
+      <c r="S35" t="n">
+        <v>6</v>
+      </c>
+      <c r="T35" t="n">
+        <v>1</v>
+      </c>
+      <c r="U35" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2888,6 +3518,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G39" t="n">
+        <v>11</v>
+      </c>
+      <c r="H39" t="n">
+        <v>10</v>
+      </c>
+      <c r="I39" t="n">
+        <v>21</v>
+      </c>
+      <c r="J39" t="n">
+        <v>11</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" t="n">
+        <v>12</v>
+      </c>
+      <c r="M39" t="n">
+        <v>3</v>
+      </c>
+      <c r="N39" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" t="n">
+        <v>4</v>
+      </c>
+      <c r="P39" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>11</v>
+      </c>
+      <c r="R39" t="n">
+        <v>37</v>
+      </c>
+      <c r="S39" t="n">
+        <v>7</v>
+      </c>
+      <c r="T39" t="n">
+        <v>3</v>
+      </c>
+      <c r="U39" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2920,6 +3595,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G40" t="n">
+        <v>17</v>
+      </c>
+      <c r="H40" t="n">
+        <v>11</v>
+      </c>
+      <c r="I40" t="n">
+        <v>28</v>
+      </c>
+      <c r="J40" t="n">
+        <v>6</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" t="n">
+        <v>7</v>
+      </c>
+      <c r="M40" t="n">
+        <v>2</v>
+      </c>
+      <c r="N40" t="n">
+        <v>3</v>
+      </c>
+      <c r="O40" t="n">
+        <v>5</v>
+      </c>
+      <c r="P40" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>5</v>
+      </c>
+      <c r="R40" t="n">
+        <v>20</v>
+      </c>
+      <c r="S40" t="n">
+        <v>6</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1</v>
+      </c>
+      <c r="U40" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2952,6 +3672,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G41" t="n">
+        <v>13</v>
+      </c>
+      <c r="H41" t="n">
+        <v>13</v>
+      </c>
+      <c r="I41" t="n">
+        <v>26</v>
+      </c>
+      <c r="J41" t="n">
+        <v>9</v>
+      </c>
+      <c r="K41" t="n">
+        <v>7</v>
+      </c>
+      <c r="L41" t="n">
+        <v>16</v>
+      </c>
+      <c r="M41" t="n">
+        <v>1</v>
+      </c>
+      <c r="N41" t="n">
+        <v>2</v>
+      </c>
+      <c r="O41" t="n">
+        <v>3</v>
+      </c>
+      <c r="P41" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>16</v>
+      </c>
+      <c r="R41" t="n">
+        <v>24</v>
+      </c>
+      <c r="S41" t="n">
+        <v>3</v>
+      </c>
+      <c r="T41" t="n">
+        <v>4</v>
+      </c>
+      <c r="U41" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2984,6 +3749,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G42" t="n">
+        <v>9</v>
+      </c>
+      <c r="H42" t="n">
+        <v>16</v>
+      </c>
+      <c r="I42" t="n">
+        <v>25</v>
+      </c>
+      <c r="J42" t="n">
+        <v>8</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1</v>
+      </c>
+      <c r="L42" t="n">
+        <v>9</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" t="n">
+        <v>1</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2</v>
+      </c>
+      <c r="P42" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>8</v>
+      </c>
+      <c r="R42" t="n">
+        <v>22</v>
+      </c>
+      <c r="S42" t="n">
+        <v>4</v>
+      </c>
+      <c r="T42" t="n">
+        <v>2</v>
+      </c>
+      <c r="U42" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3016,6 +3826,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G43" t="n">
+        <v>9</v>
+      </c>
+      <c r="H43" t="n">
+        <v>12</v>
+      </c>
+      <c r="I43" t="n">
+        <v>21</v>
+      </c>
+      <c r="J43" t="n">
+        <v>4</v>
+      </c>
+      <c r="K43" t="n">
+        <v>5</v>
+      </c>
+      <c r="L43" t="n">
+        <v>9</v>
+      </c>
+      <c r="M43" t="n">
+        <v>3</v>
+      </c>
+      <c r="N43" t="n">
+        <v>3</v>
+      </c>
+      <c r="O43" t="n">
+        <v>6</v>
+      </c>
+      <c r="P43" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>8</v>
+      </c>
+      <c r="R43" t="n">
+        <v>24</v>
+      </c>
+      <c r="S43" t="n">
+        <v>8</v>
+      </c>
+      <c r="T43" t="n">
+        <v>4</v>
+      </c>
+      <c r="U43" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3048,6 +3903,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G44" t="n">
+        <v>14</v>
+      </c>
+      <c r="H44" t="n">
+        <v>11</v>
+      </c>
+      <c r="I44" t="n">
+        <v>25</v>
+      </c>
+      <c r="J44" t="n">
+        <v>4</v>
+      </c>
+      <c r="K44" t="n">
+        <v>7</v>
+      </c>
+      <c r="L44" t="n">
+        <v>11</v>
+      </c>
+      <c r="M44" t="n">
+        <v>2</v>
+      </c>
+      <c r="N44" t="n">
+        <v>1</v>
+      </c>
+      <c r="O44" t="n">
+        <v>3</v>
+      </c>
+      <c r="P44" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>9</v>
+      </c>
+      <c r="R44" t="n">
+        <v>13</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1</v>
+      </c>
+      <c r="T44" t="n">
+        <v>4</v>
+      </c>
+      <c r="U44" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3080,6 +3980,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G45" t="n">
+        <v>10</v>
+      </c>
+      <c r="H45" t="n">
+        <v>9</v>
+      </c>
+      <c r="I45" t="n">
+        <v>19</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="n">
+        <v>6</v>
+      </c>
+      <c r="L45" t="n">
+        <v>7</v>
+      </c>
+      <c r="M45" t="n">
+        <v>2</v>
+      </c>
+      <c r="N45" t="n">
+        <v>1</v>
+      </c>
+      <c r="O45" t="n">
+        <v>3</v>
+      </c>
+      <c r="P45" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>20</v>
+      </c>
+      <c r="R45" t="n">
+        <v>28</v>
+      </c>
+      <c r="S45" t="n">
+        <v>4</v>
+      </c>
+      <c r="T45" t="n">
+        <v>6</v>
+      </c>
+      <c r="U45" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3112,6 +4057,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G46" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" t="n">
+        <v>15</v>
+      </c>
+      <c r="I46" t="n">
+        <v>20</v>
+      </c>
+      <c r="J46" t="n">
+        <v>4</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>4</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1</v>
+      </c>
+      <c r="O46" t="n">
+        <v>1</v>
+      </c>
+      <c r="P46" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>11</v>
+      </c>
+      <c r="R46" t="n">
+        <v>27</v>
+      </c>
+      <c r="S46" t="n">
+        <v>5</v>
+      </c>
+      <c r="T46" t="n">
+        <v>4</v>
+      </c>
+      <c r="U46" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3144,6 +4134,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G47" t="n">
+        <v>12</v>
+      </c>
+      <c r="H47" t="n">
+        <v>14</v>
+      </c>
+      <c r="I47" t="n">
+        <v>26</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>5</v>
+      </c>
+      <c r="L47" t="n">
+        <v>8</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
+        <v>3</v>
+      </c>
+      <c r="O47" t="n">
+        <v>3</v>
+      </c>
+      <c r="P47" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>11</v>
+      </c>
+      <c r="R47" t="n">
+        <v>21</v>
+      </c>
+      <c r="S47" t="n">
+        <v>3</v>
+      </c>
+      <c r="T47" t="n">
+        <v>4</v>
+      </c>
+      <c r="U47" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3176,6 +4211,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G48" t="n">
+        <v>15</v>
+      </c>
+      <c r="H48" t="n">
+        <v>14</v>
+      </c>
+      <c r="I48" t="n">
+        <v>29</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2</v>
+      </c>
+      <c r="L48" t="n">
+        <v>5</v>
+      </c>
+      <c r="M48" t="n">
+        <v>2</v>
+      </c>
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
+      <c r="O48" t="n">
+        <v>3</v>
+      </c>
+      <c r="P48" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>7</v>
+      </c>
+      <c r="R48" t="n">
+        <v>16</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2</v>
+      </c>
+      <c r="T48" t="n">
+        <v>3</v>
+      </c>
+      <c r="U48" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3208,6 +4288,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G49" t="n">
+        <v>17</v>
+      </c>
+      <c r="H49" t="n">
+        <v>14</v>
+      </c>
+      <c r="I49" t="n">
+        <v>31</v>
+      </c>
+      <c r="J49" t="n">
+        <v>7</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
+      </c>
+      <c r="L49" t="n">
+        <v>10</v>
+      </c>
+      <c r="M49" t="n">
+        <v>1</v>
+      </c>
+      <c r="N49" t="n">
+        <v>1</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2</v>
+      </c>
+      <c r="P49" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>9</v>
+      </c>
+      <c r="R49" t="n">
+        <v>35</v>
+      </c>
+      <c r="S49" t="n">
+        <v>8</v>
+      </c>
+      <c r="T49" t="n">
+        <v>4</v>
+      </c>
+      <c r="U49" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3240,6 +4365,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G50" t="n">
+        <v>11</v>
+      </c>
+      <c r="H50" t="n">
+        <v>17</v>
+      </c>
+      <c r="I50" t="n">
+        <v>28</v>
+      </c>
+      <c r="J50" t="n">
+        <v>9</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" t="n">
+        <v>10</v>
+      </c>
+      <c r="M50" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" t="n">
+        <v>3</v>
+      </c>
+      <c r="O50" t="n">
+        <v>4</v>
+      </c>
+      <c r="P50" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>7</v>
+      </c>
+      <c r="R50" t="n">
+        <v>25</v>
+      </c>
+      <c r="S50" t="n">
+        <v>5</v>
+      </c>
+      <c r="T50" t="n">
+        <v>3</v>
+      </c>
+      <c r="U50" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3272,6 +4442,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G51" t="n">
+        <v>17</v>
+      </c>
+      <c r="H51" t="n">
+        <v>17</v>
+      </c>
+      <c r="I51" t="n">
+        <v>34</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="n">
+        <v>2</v>
+      </c>
+      <c r="L51" t="n">
+        <v>3</v>
+      </c>
+      <c r="M51" t="n">
+        <v>2</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3</v>
+      </c>
+      <c r="O51" t="n">
+        <v>5</v>
+      </c>
+      <c r="P51" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>5</v>
+      </c>
+      <c r="R51" t="n">
+        <v>11</v>
+      </c>
+      <c r="S51" t="n">
+        <v>2</v>
+      </c>
+      <c r="T51" t="n">
+        <v>3</v>
+      </c>
+      <c r="U51" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3304,6 +4519,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G52" t="n">
+        <v>2</v>
+      </c>
+      <c r="H52" t="n">
+        <v>6</v>
+      </c>
+      <c r="I52" t="n">
+        <v>8</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>7</v>
+      </c>
+      <c r="L52" t="n">
+        <v>7</v>
+      </c>
+      <c r="M52" t="n">
+        <v>5</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" t="n">
+        <v>6</v>
+      </c>
+      <c r="P52" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>11</v>
+      </c>
+      <c r="R52" t="n">
+        <v>13</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1</v>
+      </c>
+      <c r="T52" t="n">
+        <v>7</v>
+      </c>
+      <c r="U52" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3336,6 +4596,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G53" t="n">
+        <v>5</v>
+      </c>
+      <c r="H53" t="n">
+        <v>14</v>
+      </c>
+      <c r="I53" t="n">
+        <v>19</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" t="n">
+        <v>6</v>
+      </c>
+      <c r="M53" t="n">
+        <v>2</v>
+      </c>
+      <c r="N53" t="n">
+        <v>2</v>
+      </c>
+      <c r="O53" t="n">
+        <v>4</v>
+      </c>
+      <c r="P53" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>7</v>
+      </c>
+      <c r="R53" t="n">
+        <v>20</v>
+      </c>
+      <c r="S53" t="n">
+        <v>5</v>
+      </c>
+      <c r="T53" t="n">
+        <v>3</v>
+      </c>
+      <c r="U53" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3368,6 +4673,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G54" t="n">
+        <v>13</v>
+      </c>
+      <c r="H54" t="n">
+        <v>11</v>
+      </c>
+      <c r="I54" t="n">
+        <v>24</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" t="n">
+        <v>10</v>
+      </c>
+      <c r="L54" t="n">
+        <v>11</v>
+      </c>
+      <c r="M54" t="n">
+        <v>3</v>
+      </c>
+      <c r="N54" t="n">
+        <v>2</v>
+      </c>
+      <c r="O54" t="n">
+        <v>5</v>
+      </c>
+      <c r="P54" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>20</v>
+      </c>
+      <c r="R54" t="n">
+        <v>37</v>
+      </c>
+      <c r="S54" t="n">
+        <v>3</v>
+      </c>
+      <c r="T54" t="n">
+        <v>6</v>
+      </c>
+      <c r="U54" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3400,6 +4750,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H55" t="n">
+        <v>7</v>
+      </c>
+      <c r="I55" t="n">
+        <v>17</v>
+      </c>
+      <c r="J55" t="n">
+        <v>5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>5</v>
+      </c>
+      <c r="L55" t="n">
+        <v>10</v>
+      </c>
+      <c r="M55" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" t="n">
+        <v>1</v>
+      </c>
+      <c r="O55" t="n">
+        <v>2</v>
+      </c>
+      <c r="P55" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>13</v>
+      </c>
+      <c r="R55" t="n">
+        <v>24</v>
+      </c>
+      <c r="S55" t="n">
+        <v>2</v>
+      </c>
+      <c r="T55" t="n">
+        <v>4</v>
+      </c>
+      <c r="U55" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3432,6 +4827,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G56" t="n">
+        <v>6</v>
+      </c>
+      <c r="H56" t="n">
+        <v>20</v>
+      </c>
+      <c r="I56" t="n">
+        <v>26</v>
+      </c>
+      <c r="J56" t="n">
+        <v>3</v>
+      </c>
+      <c r="K56" t="n">
+        <v>2</v>
+      </c>
+      <c r="L56" t="n">
+        <v>5</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="n">
+        <v>2</v>
+      </c>
+      <c r="O56" t="n">
+        <v>2</v>
+      </c>
+      <c r="P56" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>14</v>
+      </c>
+      <c r="R56" t="n">
+        <v>27</v>
+      </c>
+      <c r="S56" t="n">
+        <v>2</v>
+      </c>
+      <c r="T56" t="n">
+        <v>5</v>
+      </c>
+      <c r="U56" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3464,6 +4904,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G57" t="n">
+        <v>9</v>
+      </c>
+      <c r="H57" t="n">
+        <v>11</v>
+      </c>
+      <c r="I57" t="n">
+        <v>20</v>
+      </c>
+      <c r="J57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" t="n">
+        <v>15</v>
+      </c>
+      <c r="L57" t="n">
+        <v>16</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" t="n">
+        <v>1</v>
+      </c>
+      <c r="O57" t="n">
+        <v>1</v>
+      </c>
+      <c r="P57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>19</v>
+      </c>
+      <c r="R57" t="n">
+        <v>22</v>
+      </c>
+      <c r="S57" t="n">
+        <v>2</v>
+      </c>
+      <c r="T57" t="n">
+        <v>10</v>
+      </c>
+      <c r="U57" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3496,6 +4981,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G58" t="n">
+        <v>10</v>
+      </c>
+      <c r="H58" t="n">
+        <v>13</v>
+      </c>
+      <c r="I58" t="n">
+        <v>23</v>
+      </c>
+      <c r="J58" t="n">
+        <v>5</v>
+      </c>
+      <c r="K58" t="n">
+        <v>7</v>
+      </c>
+      <c r="L58" t="n">
+        <v>12</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>16</v>
+      </c>
+      <c r="R58" t="n">
+        <v>30</v>
+      </c>
+      <c r="S58" t="n">
+        <v>6</v>
+      </c>
+      <c r="T58" t="n">
+        <v>4</v>
+      </c>
+      <c r="U58" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3528,6 +5058,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G59" t="n">
+        <v>6</v>
+      </c>
+      <c r="H59" t="n">
+        <v>13</v>
+      </c>
+      <c r="I59" t="n">
+        <v>19</v>
+      </c>
+      <c r="J59" t="n">
+        <v>5</v>
+      </c>
+      <c r="K59" t="n">
+        <v>3</v>
+      </c>
+      <c r="L59" t="n">
+        <v>8</v>
+      </c>
+      <c r="M59" t="n">
+        <v>1</v>
+      </c>
+      <c r="N59" t="n">
+        <v>2</v>
+      </c>
+      <c r="O59" t="n">
+        <v>3</v>
+      </c>
+      <c r="P59" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>20</v>
+      </c>
+      <c r="R59" t="n">
+        <v>38</v>
+      </c>
+      <c r="S59" t="n">
+        <v>0</v>
+      </c>
+      <c r="T59" t="n">
+        <v>2</v>
+      </c>
+      <c r="U59" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3560,6 +5135,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G60" t="n">
+        <v>8</v>
+      </c>
+      <c r="H60" t="n">
+        <v>8</v>
+      </c>
+      <c r="I60" t="n">
+        <v>16</v>
+      </c>
+      <c r="J60" t="n">
+        <v>3</v>
+      </c>
+      <c r="K60" t="n">
+        <v>10</v>
+      </c>
+      <c r="L60" t="n">
+        <v>13</v>
+      </c>
+      <c r="M60" t="n">
+        <v>1</v>
+      </c>
+      <c r="N60" t="n">
+        <v>1</v>
+      </c>
+      <c r="O60" t="n">
+        <v>2</v>
+      </c>
+      <c r="P60" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>24</v>
+      </c>
+      <c r="R60" t="n">
+        <v>44</v>
+      </c>
+      <c r="S60" t="n">
+        <v>7</v>
+      </c>
+      <c r="T60" t="n">
+        <v>7</v>
+      </c>
+      <c r="U60" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3592,6 +5212,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G61" t="n">
+        <v>11</v>
+      </c>
+      <c r="H61" t="n">
+        <v>19</v>
+      </c>
+      <c r="I61" t="n">
+        <v>30</v>
+      </c>
+      <c r="J61" t="n">
+        <v>7</v>
+      </c>
+      <c r="K61" t="n">
+        <v>2</v>
+      </c>
+      <c r="L61" t="n">
+        <v>9</v>
+      </c>
+      <c r="M61" t="n">
+        <v>2</v>
+      </c>
+      <c r="N61" t="n">
+        <v>4</v>
+      </c>
+      <c r="O61" t="n">
+        <v>6</v>
+      </c>
+      <c r="P61" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>5</v>
+      </c>
+      <c r="R61" t="n">
+        <v>21</v>
+      </c>
+      <c r="S61" t="n">
+        <v>6</v>
+      </c>
+      <c r="T61" t="n">
+        <v>1</v>
+      </c>
+      <c r="U61" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3624,6 +5289,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G62" t="n">
+        <v>17</v>
+      </c>
+      <c r="H62" t="n">
+        <v>12</v>
+      </c>
+      <c r="I62" t="n">
+        <v>29</v>
+      </c>
+      <c r="J62" t="n">
+        <v>4</v>
+      </c>
+      <c r="K62" t="n">
+        <v>6</v>
+      </c>
+      <c r="L62" t="n">
+        <v>10</v>
+      </c>
+      <c r="M62" t="n">
+        <v>5</v>
+      </c>
+      <c r="N62" t="n">
+        <v>6</v>
+      </c>
+      <c r="O62" t="n">
+        <v>11</v>
+      </c>
+      <c r="P62" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>12</v>
+      </c>
+      <c r="R62" t="n">
+        <v>24</v>
+      </c>
+      <c r="S62" t="n">
+        <v>5</v>
+      </c>
+      <c r="T62" t="n">
+        <v>6</v>
+      </c>
+      <c r="U62" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3656,6 +5366,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G63" t="n">
+        <v>14</v>
+      </c>
+      <c r="H63" t="n">
+        <v>9</v>
+      </c>
+      <c r="I63" t="n">
+        <v>23</v>
+      </c>
+      <c r="J63" t="n">
+        <v>6</v>
+      </c>
+      <c r="K63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L63" t="n">
+        <v>8</v>
+      </c>
+      <c r="M63" t="n">
+        <v>2</v>
+      </c>
+      <c r="N63" t="n">
+        <v>3</v>
+      </c>
+      <c r="O63" t="n">
+        <v>5</v>
+      </c>
+      <c r="P63" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>9</v>
+      </c>
+      <c r="R63" t="n">
+        <v>29</v>
+      </c>
+      <c r="S63" t="n">
+        <v>7</v>
+      </c>
+      <c r="T63" t="n">
+        <v>0</v>
+      </c>
+      <c r="U63" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3688,6 +5443,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G64" t="n">
+        <v>11</v>
+      </c>
+      <c r="H64" t="n">
+        <v>11</v>
+      </c>
+      <c r="I64" t="n">
+        <v>22</v>
+      </c>
+      <c r="J64" t="n">
+        <v>8</v>
+      </c>
+      <c r="K64" t="n">
+        <v>3</v>
+      </c>
+      <c r="L64" t="n">
+        <v>11</v>
+      </c>
+      <c r="M64" t="n">
+        <v>1</v>
+      </c>
+      <c r="N64" t="n">
+        <v>2</v>
+      </c>
+      <c r="O64" t="n">
+        <v>3</v>
+      </c>
+      <c r="P64" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>5</v>
+      </c>
+      <c r="R64" t="n">
+        <v>19</v>
+      </c>
+      <c r="S64" t="n">
+        <v>6</v>
+      </c>
+      <c r="T64" t="n">
+        <v>4</v>
+      </c>
+      <c r="U64" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3720,6 +5520,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G65" t="n">
+        <v>16</v>
+      </c>
+      <c r="H65" t="n">
+        <v>15</v>
+      </c>
+      <c r="I65" t="n">
+        <v>31</v>
+      </c>
+      <c r="J65" t="n">
+        <v>2</v>
+      </c>
+      <c r="K65" t="n">
+        <v>6</v>
+      </c>
+      <c r="L65" t="n">
+        <v>8</v>
+      </c>
+      <c r="M65" t="n">
+        <v>5</v>
+      </c>
+      <c r="N65" t="n">
+        <v>3</v>
+      </c>
+      <c r="O65" t="n">
+        <v>8</v>
+      </c>
+      <c r="P65" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>27</v>
+      </c>
+      <c r="R65" t="n">
+        <v>40</v>
+      </c>
+      <c r="S65" t="n">
+        <v>4</v>
+      </c>
+      <c r="T65" t="n">
+        <v>7</v>
+      </c>
+      <c r="U65" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3752,6 +5597,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G66" t="n">
+        <v>10</v>
+      </c>
+      <c r="H66" t="n">
+        <v>13</v>
+      </c>
+      <c r="I66" t="n">
+        <v>23</v>
+      </c>
+      <c r="J66" t="n">
+        <v>2</v>
+      </c>
+      <c r="K66" t="n">
+        <v>3</v>
+      </c>
+      <c r="L66" t="n">
+        <v>5</v>
+      </c>
+      <c r="M66" t="n">
+        <v>2</v>
+      </c>
+      <c r="N66" t="n">
+        <v>2</v>
+      </c>
+      <c r="O66" t="n">
+        <v>4</v>
+      </c>
+      <c r="P66" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>6</v>
+      </c>
+      <c r="R66" t="n">
+        <v>17</v>
+      </c>
+      <c r="S66" t="n">
+        <v>2</v>
+      </c>
+      <c r="T66" t="n">
+        <v>7</v>
+      </c>
+      <c r="U66" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3784,6 +5674,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G67" t="n">
+        <v>14</v>
+      </c>
+      <c r="H67" t="n">
+        <v>17</v>
+      </c>
+      <c r="I67" t="n">
+        <v>31</v>
+      </c>
+      <c r="J67" t="n">
+        <v>8</v>
+      </c>
+      <c r="K67" t="n">
+        <v>6</v>
+      </c>
+      <c r="L67" t="n">
+        <v>14</v>
+      </c>
+      <c r="M67" t="n">
+        <v>1</v>
+      </c>
+      <c r="N67" t="n">
+        <v>3</v>
+      </c>
+      <c r="O67" t="n">
+        <v>4</v>
+      </c>
+      <c r="P67" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>6</v>
+      </c>
+      <c r="R67" t="n">
+        <v>18</v>
+      </c>
+      <c r="S67" t="n">
+        <v>1</v>
+      </c>
+      <c r="T67" t="n">
+        <v>3</v>
+      </c>
+      <c r="U67" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3816,6 +5751,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G68" t="n">
+        <v>11</v>
+      </c>
+      <c r="H68" t="n">
+        <v>12</v>
+      </c>
+      <c r="I68" t="n">
+        <v>23</v>
+      </c>
+      <c r="J68" t="n">
+        <v>3</v>
+      </c>
+      <c r="K68" t="n">
+        <v>1</v>
+      </c>
+      <c r="L68" t="n">
+        <v>4</v>
+      </c>
+      <c r="M68" t="n">
+        <v>1</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
+        <v>1</v>
+      </c>
+      <c r="P68" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>12</v>
+      </c>
+      <c r="R68" t="n">
+        <v>19</v>
+      </c>
+      <c r="S68" t="n">
+        <v>2</v>
+      </c>
+      <c r="T68" t="n">
+        <v>7</v>
+      </c>
+      <c r="U68" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3848,6 +5828,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G69" t="n">
+        <v>15</v>
+      </c>
+      <c r="H69" t="n">
+        <v>18</v>
+      </c>
+      <c r="I69" t="n">
+        <v>33</v>
+      </c>
+      <c r="J69" t="n">
+        <v>3</v>
+      </c>
+      <c r="K69" t="n">
+        <v>12</v>
+      </c>
+      <c r="L69" t="n">
+        <v>15</v>
+      </c>
+      <c r="M69" t="n">
+        <v>2</v>
+      </c>
+      <c r="N69" t="n">
+        <v>2</v>
+      </c>
+      <c r="O69" t="n">
+        <v>4</v>
+      </c>
+      <c r="P69" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>19</v>
+      </c>
+      <c r="R69" t="n">
+        <v>30</v>
+      </c>
+      <c r="S69" t="n">
+        <v>2</v>
+      </c>
+      <c r="T69" t="n">
+        <v>5</v>
+      </c>
+      <c r="U69" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3880,6 +5905,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G70" t="n">
+        <v>8</v>
+      </c>
+      <c r="H70" t="n">
+        <v>12</v>
+      </c>
+      <c r="I70" t="n">
+        <v>20</v>
+      </c>
+      <c r="J70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L70" t="n">
+        <v>8</v>
+      </c>
+      <c r="M70" t="n">
+        <v>1</v>
+      </c>
+      <c r="N70" t="n">
+        <v>3</v>
+      </c>
+      <c r="O70" t="n">
+        <v>4</v>
+      </c>
+      <c r="P70" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>12</v>
+      </c>
+      <c r="R70" t="n">
+        <v>31</v>
+      </c>
+      <c r="S70" t="n">
+        <v>7</v>
+      </c>
+      <c r="T70" t="n">
+        <v>5</v>
+      </c>
+      <c r="U70" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3912,6 +5982,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G71" t="n">
+        <v>9</v>
+      </c>
+      <c r="H71" t="n">
+        <v>10</v>
+      </c>
+      <c r="I71" t="n">
+        <v>19</v>
+      </c>
+      <c r="J71" t="n">
+        <v>4</v>
+      </c>
+      <c r="K71" t="n">
+        <v>4</v>
+      </c>
+      <c r="L71" t="n">
+        <v>8</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>22</v>
+      </c>
+      <c r="R71" t="n">
+        <v>36</v>
+      </c>
+      <c r="S71" t="n">
+        <v>7</v>
+      </c>
+      <c r="T71" t="n">
+        <v>8</v>
+      </c>
+      <c r="U71" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3944,6 +6059,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G72" t="n">
+        <v>10</v>
+      </c>
+      <c r="H72" t="n">
+        <v>9</v>
+      </c>
+      <c r="I72" t="n">
+        <v>19</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" t="n">
+        <v>4</v>
+      </c>
+      <c r="L72" t="n">
+        <v>6</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="n">
+        <v>1</v>
+      </c>
+      <c r="O72" t="n">
+        <v>1</v>
+      </c>
+      <c r="P72" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>19</v>
+      </c>
+      <c r="R72" t="n">
+        <v>27</v>
+      </c>
+      <c r="S72" t="n">
+        <v>1</v>
+      </c>
+      <c r="T72" t="n">
+        <v>4</v>
+      </c>
+      <c r="U72" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3976,6 +6136,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G73" t="n">
+        <v>10</v>
+      </c>
+      <c r="H73" t="n">
+        <v>13</v>
+      </c>
+      <c r="I73" t="n">
+        <v>23</v>
+      </c>
+      <c r="J73" t="n">
+        <v>5</v>
+      </c>
+      <c r="K73" t="n">
+        <v>3</v>
+      </c>
+      <c r="L73" t="n">
+        <v>8</v>
+      </c>
+      <c r="M73" t="n">
+        <v>1</v>
+      </c>
+      <c r="N73" t="n">
+        <v>2</v>
+      </c>
+      <c r="O73" t="n">
+        <v>3</v>
+      </c>
+      <c r="P73" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>16</v>
+      </c>
+      <c r="R73" t="n">
+        <v>27</v>
+      </c>
+      <c r="S73" t="n">
+        <v>2</v>
+      </c>
+      <c r="T73" t="n">
+        <v>1</v>
+      </c>
+      <c r="U73" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4008,6 +6213,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G74" t="n">
+        <v>10</v>
+      </c>
+      <c r="H74" t="n">
+        <v>3</v>
+      </c>
+      <c r="I74" t="n">
+        <v>13</v>
+      </c>
+      <c r="J74" t="n">
+        <v>9</v>
+      </c>
+      <c r="K74" t="n">
+        <v>4</v>
+      </c>
+      <c r="L74" t="n">
+        <v>13</v>
+      </c>
+      <c r="M74" t="n">
+        <v>1</v>
+      </c>
+      <c r="N74" t="n">
+        <v>1</v>
+      </c>
+      <c r="O74" t="n">
+        <v>2</v>
+      </c>
+      <c r="P74" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>3</v>
+      </c>
+      <c r="R74" t="n">
+        <v>28</v>
+      </c>
+      <c r="S74" t="n">
+        <v>12</v>
+      </c>
+      <c r="T74" t="n">
+        <v>2</v>
+      </c>
+      <c r="U74" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4040,6 +6290,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G75" t="n">
+        <v>14</v>
+      </c>
+      <c r="H75" t="n">
+        <v>13</v>
+      </c>
+      <c r="I75" t="n">
+        <v>27</v>
+      </c>
+      <c r="J75" t="n">
+        <v>3</v>
+      </c>
+      <c r="K75" t="n">
+        <v>3</v>
+      </c>
+      <c r="L75" t="n">
+        <v>6</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>1</v>
+      </c>
+      <c r="O75" t="n">
+        <v>1</v>
+      </c>
+      <c r="P75" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>14</v>
+      </c>
+      <c r="R75" t="n">
+        <v>25</v>
+      </c>
+      <c r="S75" t="n">
+        <v>1</v>
+      </c>
+      <c r="T75" t="n">
+        <v>2</v>
+      </c>
+      <c r="U75" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4072,6 +6367,51 @@
           <t>так</t>
         </is>
       </c>
+      <c r="G76" t="n">
+        <v>14</v>
+      </c>
+      <c r="H76" t="n">
+        <v>16</v>
+      </c>
+      <c r="I76" t="n">
+        <v>30</v>
+      </c>
+      <c r="J76" t="n">
+        <v>9</v>
+      </c>
+      <c r="K76" t="n">
+        <v>5</v>
+      </c>
+      <c r="L76" t="n">
+        <v>14</v>
+      </c>
+      <c r="M76" t="n">
+        <v>2</v>
+      </c>
+      <c r="N76" t="n">
+        <v>3</v>
+      </c>
+      <c r="O76" t="n">
+        <v>5</v>
+      </c>
+      <c r="P76" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>12</v>
+      </c>
+      <c r="R76" t="n">
+        <v>36</v>
+      </c>
+      <c r="S76" t="n">
+        <v>6</v>
+      </c>
+      <c r="T76" t="n">
+        <v>5</v>
+      </c>
+      <c r="U76" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4104,6 +6444,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G77" t="n">
+        <v>14</v>
+      </c>
+      <c r="H77" t="n">
+        <v>13</v>
+      </c>
+      <c r="I77" t="n">
+        <v>27</v>
+      </c>
+      <c r="J77" t="n">
+        <v>5</v>
+      </c>
+      <c r="K77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L77" t="n">
+        <v>7</v>
+      </c>
+      <c r="M77" t="n">
+        <v>2</v>
+      </c>
+      <c r="N77" t="n">
+        <v>1</v>
+      </c>
+      <c r="O77" t="n">
+        <v>3</v>
+      </c>
+      <c r="P77" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>17</v>
+      </c>
+      <c r="R77" t="n">
+        <v>26</v>
+      </c>
+      <c r="S77" t="n">
+        <v>2</v>
+      </c>
+      <c r="T77" t="n">
+        <v>5</v>
+      </c>
+      <c r="U77" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4136,6 +6521,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G78" t="n">
+        <v>18</v>
+      </c>
+      <c r="H78" t="n">
+        <v>12</v>
+      </c>
+      <c r="I78" t="n">
+        <v>30</v>
+      </c>
+      <c r="J78" t="n">
+        <v>5</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>5</v>
+      </c>
+      <c r="M78" t="n">
+        <v>1</v>
+      </c>
+      <c r="N78" t="n">
+        <v>1</v>
+      </c>
+      <c r="O78" t="n">
+        <v>2</v>
+      </c>
+      <c r="P78" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>8</v>
+      </c>
+      <c r="R78" t="n">
+        <v>21</v>
+      </c>
+      <c r="S78" t="n">
+        <v>4</v>
+      </c>
+      <c r="T78" t="n">
+        <v>3</v>
+      </c>
+      <c r="U78" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4168,6 +6598,51 @@
           <t>ні</t>
         </is>
       </c>
+      <c r="G79" t="n">
+        <v>12</v>
+      </c>
+      <c r="H79" t="n">
+        <v>18</v>
+      </c>
+      <c r="I79" t="n">
+        <v>30</v>
+      </c>
+      <c r="J79" t="n">
+        <v>8</v>
+      </c>
+      <c r="K79" t="n">
+        <v>1</v>
+      </c>
+      <c r="L79" t="n">
+        <v>9</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>2</v>
+      </c>
+      <c r="O79" t="n">
+        <v>2</v>
+      </c>
+      <c r="P79" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>9</v>
+      </c>
+      <c r="R79" t="n">
+        <v>37</v>
+      </c>
+      <c r="S79" t="n">
+        <v>7</v>
+      </c>
+      <c r="T79" t="n">
+        <v>1</v>
+      </c>
+      <c r="U79" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4199,6 +6674,51 @@
         <is>
           <t>так</t>
         </is>
+      </c>
+      <c r="G80" t="n">
+        <v>11</v>
+      </c>
+      <c r="H80" t="n">
+        <v>12</v>
+      </c>
+      <c r="I80" t="n">
+        <v>23</v>
+      </c>
+      <c r="J80" t="n">
+        <v>6</v>
+      </c>
+      <c r="K80" t="n">
+        <v>4</v>
+      </c>
+      <c r="L80" t="n">
+        <v>10</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>4</v>
+      </c>
+      <c r="O80" t="n">
+        <v>4</v>
+      </c>
+      <c r="P80" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>9</v>
+      </c>
+      <c r="R80" t="n">
+        <v>26</v>
+      </c>
+      <c r="S80" t="n">
+        <v>8</v>
+      </c>
+      <c r="T80" t="n">
+        <v>4</v>
+      </c>
+      <c r="U80" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>